<commit_message>
Update test generators to strictly include Selenium, Appium, Unit, Security, Vulnerability and Load Testing
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Target URL: https://madhanr13.github.io/Snap-Solve/ | Generated: 2026-07-27 13:21:23 | Total Test Cases: 0</t>
+          <t>Target URL: https://madhanr13.github.io/Snap-Solve/ | Generated: 2026-07-27 13:48:44 | Total Test Cases: 0</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-27 13:21:23</t>
+          <t>2026-07-27 13:48:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: strictly limit test suite cases to 300 per suite
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Target URL: https://madhanr13.github.io/Snap-Solve/ | Generated: 2026-07-27 13:48:44 | Total Test Cases: 0</t>
+          <t>Target URL: https://madhanr13.github.io/Snap-Solve/ | Generated: 2026-07-27 14:05:04 | Total Test Cases: 0</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-27 13:48:44</t>
+          <t>2026-07-27 14:05:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restore syntax error and correctly restrict all suites to 300 test cases
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Target URL: https://madhanr13.github.io/Snap-Solve/ | Generated: 2026-07-27 14:05:04 | Total Test Cases: 0</t>
+          <t>Target URL: https://madhanr13.github.io/Snap-Solve/ | Generated: 2026-07-27 14:11:17 | Total Test Cases: 0</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-27 14:05:04</t>
+          <t>2026-07-27 14:11:17</t>
         </is>
       </c>
     </row>

</xml_diff>